<commit_message>
ATUALIZAÇÃO PLANILHA MARÇO: CHECKLIST 17/03 17h
</commit_message>
<xml_diff>
--- a/HORAS_EXTRAS_FEVEREIRO_2026.xlsx
+++ b/HORAS_EXTRAS_FEVEREIRO_2026.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projeto.dev\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8568BE3-2C40-4E54-9C3E-4F0589DBDC27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A091DF-0599-4CC7-880A-23A61D0AE4C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{7FAD56AE-9D28-4736-B635-37D3D3B1CDBF}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="45">
   <si>
     <t>HORAS EXTRAS ( FEVEREIRO / 2026 )</t>
   </si>
@@ -89,6 +89,9 @@
     <t>EDINALDO MARQUES LIMA</t>
   </si>
   <si>
+    <t>EDYMMAR UMBELINO DE OLIVEIRA</t>
+  </si>
+  <si>
     <t xml:space="preserve">OPERADOR DE VIBRO ACABADORA </t>
   </si>
   <si>
@@ -155,9 +158,6 @@
     <t>RONIELSON NASCIMENTO LIMA</t>
   </si>
   <si>
-    <t>FRANCISCO DE SOUSA SALES BOAVENTURA</t>
-  </si>
-  <si>
     <t>JOCA MARQUES</t>
   </si>
   <si>
@@ -168,6 +168,12 @@
   </si>
   <si>
     <t>JARDIM DO MULATO</t>
+  </si>
+  <si>
+    <t>NÃO COBRAR - EQUIPAMENTO USINA</t>
+  </si>
+  <si>
+    <t>FALTA LOCALIZAR O ATIVO</t>
   </si>
 </sst>
 </file>
@@ -179,7 +185,7 @@
     <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
     <numFmt numFmtId="166" formatCode="00,000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -211,6 +217,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -233,7 +246,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="3" tint="0.89999084444715716"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -283,40 +296,48 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -324,23 +345,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -687,22 +691,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" spans="1:6" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
+      <c r="A2" s="17"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="42" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -712,7 +716,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>3</v>
@@ -725,403 +729,457 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>1</v>
-      </c>
-      <c r="B4" s="3" t="s">
+      <c r="A4" s="3">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="5">
         <v>6043</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="5"/>
+      <c r="E4" s="6">
+        <v>487.19</v>
+      </c>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="14">
-        <v>2</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="9" t="s">
+      <c r="A5" s="10">
+        <v>3</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="C5" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="8"/>
+      <c r="E5" s="13">
+        <v>459</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>3</v>
-      </c>
-      <c r="B6" s="3" t="s">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="5">
         <v>6020</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="5" t="s">
+      <c r="E6" s="6">
+        <v>1561.52</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="14">
-        <v>4</v>
-      </c>
-      <c r="B7" s="6" t="s">
+      <c r="A7" s="10">
+        <v>5</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="6" t="s">
+      <c r="C7" s="12"/>
+      <c r="D7" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="8"/>
+      <c r="E7" s="13">
+        <v>425.33</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
-        <v>5</v>
-      </c>
-      <c r="B8" s="3" t="s">
+      <c r="A8" s="3">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="5">
         <v>6054</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="5"/>
+      <c r="E8" s="6">
+        <v>677.12</v>
+      </c>
+      <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="14">
+      <c r="A9" s="10">
+        <v>7</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="12"/>
+      <c r="D9" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="13">
+        <v>1184.54</v>
+      </c>
+      <c r="F9" s="14"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0</v>
+      </c>
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="10">
+        <v>9</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="12">
+        <v>6053</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" s="13">
+        <v>833.15</v>
+      </c>
+      <c r="F11" s="14"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0</v>
+      </c>
+      <c r="F12" s="7"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="10">
+        <v>11</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="12">
+        <v>2022</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="13">
+        <v>189.85</v>
+      </c>
+      <c r="F13" s="14"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="5">
+        <v>6013</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0</v>
+      </c>
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="10">
+        <v>13</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="12">
+        <v>6016</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="13">
+        <v>0</v>
+      </c>
+      <c r="F15" s="14"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>14</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="5">
+        <v>2027</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="6">
+        <v>164.6</v>
+      </c>
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="10">
+        <v>15</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="12">
+        <v>2020</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="13">
+        <v>1240.1099999999999</v>
+      </c>
+      <c r="F17" s="14"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="5">
+        <v>6048</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="6">
+        <v>0</v>
+      </c>
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="10">
+        <v>17</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="12">
+        <v>6024</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="13">
+        <v>227.66</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="5"/>
+      <c r="D20" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" s="6">
+        <v>0</v>
+      </c>
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="10">
+        <v>19</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="12">
+        <v>6023</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" s="13">
+        <v>215.98</v>
+      </c>
+      <c r="F21" s="14"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>20</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="5">
+        <v>6051</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" s="6">
+        <v>14.29</v>
+      </c>
+      <c r="F22" s="7"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="10">
+        <v>21</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="12">
+        <v>6055</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E23" s="13">
+        <v>575.54999999999995</v>
+      </c>
+      <c r="F23" s="14"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>22</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="5">
+        <v>6049</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" s="6">
+        <v>475.51</v>
+      </c>
+      <c r="F24" s="7"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="10">
+        <v>23</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C25" s="12">
+        <v>6025</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="13">
+        <v>0</v>
+      </c>
+      <c r="F25" s="14"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
+        <v>24</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="5">
+        <v>6029</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="E26" s="6">
+        <v>0</v>
+      </c>
+      <c r="F26" s="7"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="10">
+        <v>26</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" s="12">
+        <v>2032</v>
+      </c>
+      <c r="D27" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="15" t="s">
+      <c r="E27" s="13">
+        <v>1242.31</v>
+      </c>
+      <c r="F27" s="14"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C28" s="5">
+        <v>6020</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="18"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
-        <v>7</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" s="10">
-        <v>6053</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="5"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="14">
-        <v>8</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="17"/>
-      <c r="F11" s="18"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
-        <v>9</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="10">
-        <v>2022</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="5"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="14">
-        <v>10</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="C13" s="16">
-        <v>6013</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="17"/>
-      <c r="F13" s="18"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="14">
-        <v>11</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="16">
-        <v>6016</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="17"/>
-      <c r="F14" s="18"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
-        <v>12</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="14">
-        <v>13</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="16">
-        <v>2020</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="17"/>
-      <c r="F16" s="18"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
-        <v>14</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="10">
-        <v>6048</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="5"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="14">
-        <v>15</v>
-      </c>
-      <c r="B18" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" s="17"/>
-      <c r="F18" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
-        <v>16</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="5"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="14">
-        <v>17</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" s="16">
-        <v>6023</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" s="17"/>
-      <c r="F20" s="18"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
-        <v>18</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="10">
-        <v>6051</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="5"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="14">
-        <v>19</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="C22" s="16">
-        <v>6055</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E22" s="17"/>
-      <c r="F22" s="18"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
-        <v>20</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="10">
-        <v>6049</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="5"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="14">
-        <v>21</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C24" s="16">
-        <v>6025</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E24" s="17"/>
-      <c r="F24" s="18"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
-        <v>22</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C25" s="10">
-        <v>6029</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E25" s="4"/>
-      <c r="F25" s="5"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="14">
-        <v>23</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="C26" s="16">
-        <v>6017</v>
-      </c>
-      <c r="D26" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="E26" s="17"/>
-      <c r="F26" s="18"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
-        <v>24</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C27" s="10">
-        <v>2032</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E27" s="4"/>
-      <c r="F27" s="5"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="14">
-        <v>25</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" s="16">
-        <v>6020</v>
-      </c>
-      <c r="D28" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E28" s="19"/>
-      <c r="F28" s="20" t="s">
+      <c r="E28" s="6">
+        <v>42.68</v>
+      </c>
+      <c r="F28" s="9" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C29" s="11"/>
+      <c r="C29" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:F28" xr:uid="{31974592-B8CB-4C42-B44C-371B4698EC55}"/>

</xml_diff>